<commit_message>
graphiques en png (qualité à améliorer)
</commit_message>
<xml_diff>
--- a/excel/résultats.xlsx
+++ b/excel/résultats.xlsx
@@ -149,17 +149,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0\ %"/>
     <numFmt numFmtId="166" formatCode="0.00"/>
     <numFmt numFmtId="167" formatCode="0.00\ %"/>
     <numFmt numFmtId="168" formatCode="0.0\ %"/>
-    <numFmt numFmtId="169" formatCode="0\ %"/>
-    <numFmt numFmtId="170" formatCode="0.00\ %"/>
-    <numFmt numFmtId="171" formatCode="0.00E+0"/>
+    <numFmt numFmtId="169" formatCode="0.00E+0"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -215,21 +213,7 @@
     </font>
     <font>
       <sz val="12"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="13"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -283,7 +267,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -325,18 +309,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -830,11 +802,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="50450517"/>
-        <c:axId val="65418009"/>
+        <c:axId val="97839022"/>
+        <c:axId val="59265966"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="50450517"/>
+        <c:axId val="97839022"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -899,12 +871,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="65418009"/>
+        <c:crossAx val="59265966"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="65418009"/>
+        <c:axId val="59265966"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -978,7 +950,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="50450517"/>
+        <c:crossAx val="97839022"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1429,11 +1401,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="12236608"/>
-        <c:axId val="44533922"/>
+        <c:axId val="94585710"/>
+        <c:axId val="37454558"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="12236608"/>
+        <c:axId val="94585710"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1498,12 +1470,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="44533922"/>
+        <c:crossAx val="37454558"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="44533922"/>
+        <c:axId val="37454558"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1577,7 +1549,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="12236608"/>
+        <c:crossAx val="94585710"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1623,6 +1595,9 @@
             </a:pPr>
             <a:r>
               <a:rPr sz="1200" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
               </a:rPr>
@@ -1674,12 +1649,16 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="r"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
@@ -1854,12 +1833,16 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="r"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
@@ -2010,11 +1993,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="90899503"/>
-        <c:axId val="2692944"/>
+        <c:axId val="84307685"/>
+        <c:axId val="81840256"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="90899503"/>
+        <c:axId val="84307685"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2034,6 +2017,9 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr sz="900" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:rPr>
@@ -2050,7 +2036,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="0\ %" sourceLinked="1"/>
+        <c:numFmt formatCode="0\ %" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2067,18 +2053,21 @@
           <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2692944"/>
+        <c:crossAx val="81840256"/>
         <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
+        <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="2692944"/>
+        <c:axId val="81840256"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2107,6 +2096,9 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr sz="900" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:rPr>
@@ -2123,7 +2115,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="0\ %" sourceLinked="1"/>
+        <c:numFmt formatCode="0\ %" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2140,15 +2132,18 @@
           <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="90899503"/>
+        <c:crossAx val="84307685"/>
         <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
+        <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
@@ -2192,10 +2187,13 @@
             </a:pPr>
             <a:r>
               <a:rPr sz="1300" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
               </a:rPr>
-              <a:t>Effet de la taille des blocs - image de 1050x157</a:t>
+              <a:t>Effet de la taille des blocs : t = 20 fixé - image 1050x157</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -2240,12 +2238,16 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="r"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
@@ -2322,8 +2324,8 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="34938163"/>
-        <c:axId val="54528981"/>
+        <c:axId val="30331516"/>
+        <c:axId val="97602717"/>
       </c:scatterChart>
       <c:scatterChart>
         <c:scatterStyle val="lineMarker"/>
@@ -2355,12 +2357,16 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="r"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
@@ -2437,11 +2443,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="33032934"/>
-        <c:axId val="38984355"/>
+        <c:axId val="14661021"/>
+        <c:axId val="61472382"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="34938163"/>
+        <c:axId val="30331516"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2461,6 +2467,9 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr sz="900" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:rPr>
@@ -2477,7 +2486,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2494,18 +2503,21 @@
           <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="54528981"/>
+        <c:crossAx val="97602717"/>
         <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
+        <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="54528981"/>
+        <c:axId val="97602717"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2534,6 +2546,9 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr sz="900" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:rPr>
@@ -2550,7 +2565,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2567,18 +2582,21 @@
           <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="34938163"/>
+        <c:crossAx val="30331516"/>
         <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
+        <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="33032934"/>
+        <c:axId val="14661021"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2601,17 +2619,20 @@
           <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="38984355"/>
-        <c:crossBetween val="between"/>
+        <c:crossAx val="61472382"/>
+        <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="38984355"/>
+        <c:axId val="61472382"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2631,6 +2652,9 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr sz="900" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:rPr>
@@ -2647,7 +2671,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="0.00\ %" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00\ %" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2664,15 +2688,18 @@
           <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="33032934"/>
+        <c:crossAx val="14661021"/>
         <c:crosses val="max"/>
-        <c:crossBetween val="between"/>
+        <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
@@ -2716,10 +2743,13 @@
             </a:pPr>
             <a:r>
               <a:rPr sz="1300" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
               </a:rPr>
-              <a:t>Durée et taux d'erreur en fonction de t</a:t>
+              <a:t>Effet de t : blocs de 12x12, bruit de 10% - image 1800x338</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -2764,12 +2794,16 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="r"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
@@ -2882,8 +2916,8 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="86215790"/>
-        <c:axId val="27152151"/>
+        <c:axId val="17542930"/>
+        <c:axId val="78239994"/>
       </c:scatterChart>
       <c:scatterChart>
         <c:scatterStyle val="lineMarker"/>
@@ -2915,12 +2949,16 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="r"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
@@ -3033,11 +3071,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="499305"/>
-        <c:axId val="96030707"/>
+        <c:axId val="5242227"/>
+        <c:axId val="7148327"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="86215790"/>
+        <c:axId val="17542930"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3057,6 +3095,9 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr sz="900" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:rPr>
@@ -3073,7 +3114,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -3090,18 +3131,21 @@
           <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="27152151"/>
+        <c:crossAx val="78239994"/>
         <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
+        <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="27152151"/>
+        <c:axId val="78239994"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3130,6 +3174,9 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr sz="900" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:rPr>
@@ -3146,7 +3193,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="0.00\ %" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00\ %" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -3163,18 +3210,21 @@
           <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86215790"/>
+        <c:crossAx val="17542930"/>
         <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
+        <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="499305"/>
+        <c:axId val="5242227"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3197,17 +3247,20 @@
           <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="96030707"/>
-        <c:crossBetween val="between"/>
+        <c:crossAx val="7148327"/>
+        <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="96030707"/>
+        <c:axId val="7148327"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3227,6 +3280,9 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr sz="900" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:rPr>
@@ -3243,7 +3299,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -3260,15 +3316,18 @@
           <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="499305"/>
+        <c:crossAx val="5242227"/>
         <c:crosses val="max"/>
-        <c:crossBetween val="between"/>
+        <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
@@ -3298,15 +3357,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>394200</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>15840</xdr:rowOff>
+      <xdr:colOff>393480</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>81720</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>651600</xdr:colOff>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>168840</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>16560</xdr:rowOff>
+      <xdr:rowOff>6840</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3314,8 +3373,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="10049400" y="396720"/>
-        <a:ext cx="5758920" cy="3239280"/>
+        <a:off x="10048680" y="81720"/>
+        <a:ext cx="6652440" cy="3544560"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3328,15 +3387,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>469800</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>27360</xdr:rowOff>
+      <xdr:colOff>428760</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>95400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>38520</xdr:colOff>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>260280</xdr:colOff>
       <xdr:row>38</xdr:row>
-      <xdr:rowOff>27360</xdr:rowOff>
+      <xdr:rowOff>156600</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3344,8 +3403,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="10125000" y="4028040"/>
-        <a:ext cx="5758200" cy="3238200"/>
+        <a:off x="10083960" y="3714840"/>
+        <a:ext cx="6708600" cy="3680640"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3358,15 +3417,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>527040</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>95040</xdr:rowOff>
+      <xdr:colOff>384840</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>54000</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>103680</xdr:colOff>
-      <xdr:row>57</xdr:row>
-      <xdr:rowOff>95040</xdr:rowOff>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>147240</xdr:colOff>
+      <xdr:row>60</xdr:row>
+      <xdr:rowOff>6840</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3374,8 +3433,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="10182240" y="7715160"/>
-        <a:ext cx="5766120" cy="3238560"/>
+        <a:off x="10040040" y="7483680"/>
+        <a:ext cx="7327080" cy="3953160"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3387,16 +3446,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>24120</xdr:colOff>
-      <xdr:row>60</xdr:row>
-      <xdr:rowOff>61560</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>430200</xdr:colOff>
+      <xdr:row>61</xdr:row>
+      <xdr:rowOff>27720</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>281520</xdr:colOff>
-      <xdr:row>77</xdr:row>
-      <xdr:rowOff>61560</xdr:rowOff>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>340560</xdr:colOff>
+      <xdr:row>83</xdr:row>
+      <xdr:rowOff>41400</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3404,8 +3463,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="10366920" y="11491560"/>
-        <a:ext cx="5759280" cy="3238560"/>
+        <a:off x="10085400" y="11648160"/>
+        <a:ext cx="7475040" cy="4204800"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3417,16 +3476,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>1080</xdr:colOff>
-      <xdr:row>79</xdr:row>
-      <xdr:rowOff>104400</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>456480</xdr:colOff>
+      <xdr:row>84</xdr:row>
+      <xdr:rowOff>109080</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>258840</xdr:colOff>
-      <xdr:row>96</xdr:row>
-      <xdr:rowOff>105480</xdr:rowOff>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>380880</xdr:colOff>
+      <xdr:row>105</xdr:row>
+      <xdr:rowOff>20160</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3434,8 +3493,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="10343880" y="15153840"/>
-        <a:ext cx="5759640" cy="3239640"/>
+        <a:off x="10111680" y="16111080"/>
+        <a:ext cx="7489080" cy="3911760"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3644,7 +3703,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="3" width="7.02"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="3" width="8.07"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="4" width="7.9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16383" style="0" width="10.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16383" style="1" width="10.16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6464,90 +6523,90 @@
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="0" t="s">
+      <c r="A65" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B65" s="0" t="s">
+      <c r="B65" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C65" s="0" t="n">
+      <c r="C65" s="1" t="n">
         <v>1041</v>
       </c>
-      <c r="D65" s="0" t="n">
+      <c r="D65" s="1" t="n">
         <v>462</v>
       </c>
-      <c r="E65" s="0" t="n">
+      <c r="E65" s="1" t="n">
         <v>480.942</v>
       </c>
-      <c r="F65" s="0" t="n">
-        <v>12</v>
-      </c>
-      <c r="G65" s="0" t="n">
-        <v>18</v>
-      </c>
-      <c r="H65" s="0" t="n">
-        <v>19</v>
-      </c>
-      <c r="I65" s="0" t="n">
-        <v>19</v>
-      </c>
-      <c r="J65" s="11" t="n">
+      <c r="F65" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="G65" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="H65" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="I65" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="J65" s="2" t="n">
         <v>0.01</v>
       </c>
-      <c r="K65" s="12" t="n">
+      <c r="K65" s="3" t="n">
         <v>12.5707185268402</v>
       </c>
-      <c r="L65" s="12" t="n">
+      <c r="L65" s="3" t="n">
         <v>14.3072285652161</v>
       </c>
-      <c r="M65" s="13" t="n">
+      <c r="M65" s="4" t="n">
         <v>0.000110200398384836</v>
       </c>
-      <c r="N65" s="13" t="n">
+      <c r="N65" s="4" t="n">
         <v>0.000108121145585123</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="0" t="s">
+      <c r="A66" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B66" s="0" t="s">
+      <c r="B66" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C66" s="0" t="n">
+      <c r="C66" s="1" t="n">
         <v>1041</v>
       </c>
-      <c r="D66" s="0" t="n">
+      <c r="D66" s="1" t="n">
         <v>462</v>
       </c>
-      <c r="E66" s="0" t="n">
+      <c r="E66" s="1" t="n">
         <v>480.942</v>
       </c>
-      <c r="F66" s="0" t="n">
-        <v>12</v>
-      </c>
-      <c r="G66" s="0" t="n">
-        <v>18</v>
-      </c>
-      <c r="H66" s="0" t="n">
-        <v>19</v>
-      </c>
-      <c r="I66" s="0" t="n">
-        <v>19</v>
-      </c>
-      <c r="J66" s="11" t="n">
+      <c r="F66" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="G66" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="H66" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="I66" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="J66" s="2" t="n">
         <v>0.02</v>
       </c>
-      <c r="K66" s="12" t="n">
+      <c r="K66" s="3" t="n">
         <v>18.2192418575287</v>
       </c>
-      <c r="L66" s="12" t="n">
+      <c r="L66" s="3" t="n">
         <v>21.5575098991394</v>
       </c>
-      <c r="M66" s="13" t="n">
+      <c r="M66" s="4" t="n">
         <v>0.00043248458234049</v>
       </c>
-      <c r="N66" s="13" t="n">
+      <c r="N66" s="4" t="n">
         <v>0.000424167571141635</v>
       </c>
     </row>
@@ -6596,90 +6655,90 @@
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="0" t="s">
+      <c r="A68" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B68" s="0" t="s">
+      <c r="B68" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C68" s="0" t="n">
+      <c r="C68" s="1" t="n">
         <v>1041</v>
       </c>
-      <c r="D68" s="0" t="n">
+      <c r="D68" s="1" t="n">
         <v>462</v>
       </c>
-      <c r="E68" s="0" t="n">
+      <c r="E68" s="1" t="n">
         <v>480.942</v>
       </c>
-      <c r="F68" s="0" t="n">
-        <v>12</v>
-      </c>
-      <c r="G68" s="0" t="n">
-        <v>18</v>
-      </c>
-      <c r="H68" s="0" t="n">
-        <v>19</v>
-      </c>
-      <c r="I68" s="0" t="n">
-        <v>19</v>
-      </c>
-      <c r="J68" s="11" t="n">
+      <c r="F68" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="G68" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="H68" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="I68" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="J68" s="2" t="n">
         <v>0.04</v>
       </c>
-      <c r="K68" s="12" t="n">
+      <c r="K68" s="3" t="n">
         <v>18.3498024940491</v>
       </c>
-      <c r="L68" s="12" t="n">
+      <c r="L68" s="3" t="n">
         <v>26.0039048194885</v>
       </c>
-      <c r="M68" s="13" t="n">
+      <c r="M68" s="4" t="n">
         <v>0.00179855367175252</v>
       </c>
-      <c r="N68" s="13" t="n">
+      <c r="N68" s="4" t="n">
         <v>0.00170706654856511</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="0" t="s">
+      <c r="A69" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B69" s="0" t="s">
+      <c r="B69" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C69" s="0" t="n">
+      <c r="C69" s="1" t="n">
         <v>1041</v>
       </c>
-      <c r="D69" s="0" t="n">
+      <c r="D69" s="1" t="n">
         <v>462</v>
       </c>
-      <c r="E69" s="0" t="n">
+      <c r="E69" s="1" t="n">
         <v>480.942</v>
       </c>
-      <c r="F69" s="0" t="n">
-        <v>12</v>
-      </c>
-      <c r="G69" s="0" t="n">
-        <v>18</v>
-      </c>
-      <c r="H69" s="0" t="n">
-        <v>19</v>
-      </c>
-      <c r="I69" s="0" t="n">
-        <v>19</v>
-      </c>
-      <c r="J69" s="11" t="n">
+      <c r="F69" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="G69" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="H69" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="I69" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="J69" s="2" t="n">
         <v>0.05</v>
       </c>
-      <c r="K69" s="12" t="n">
+      <c r="K69" s="3" t="n">
         <v>19.6809089183807</v>
       </c>
-      <c r="L69" s="12" t="n">
+      <c r="L69" s="3" t="n">
         <v>26.8456692695618</v>
       </c>
-      <c r="M69" s="13" t="n">
+      <c r="M69" s="4" t="n">
         <v>0.00482178724253652</v>
       </c>
-      <c r="N69" s="13" t="n">
+      <c r="N69" s="4" t="n">
         <v>0.0044745520249843</v>
       </c>
     </row>
@@ -6728,90 +6787,90 @@
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="0" t="s">
+      <c r="A71" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B71" s="0" t="s">
+      <c r="B71" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C71" s="0" t="n">
+      <c r="C71" s="1" t="n">
         <v>1041</v>
       </c>
-      <c r="D71" s="0" t="n">
+      <c r="D71" s="1" t="n">
         <v>462</v>
       </c>
-      <c r="E71" s="0" t="n">
+      <c r="E71" s="1" t="n">
         <v>480.942</v>
       </c>
-      <c r="F71" s="0" t="n">
-        <v>12</v>
-      </c>
-      <c r="G71" s="0" t="n">
-        <v>18</v>
-      </c>
-      <c r="H71" s="0" t="n">
-        <v>19</v>
-      </c>
-      <c r="I71" s="0" t="n">
-        <v>19</v>
-      </c>
-      <c r="J71" s="11" t="n">
+      <c r="F71" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="G71" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="H71" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="I71" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="J71" s="2" t="n">
         <v>0.07</v>
       </c>
-      <c r="K71" s="12" t="n">
+      <c r="K71" s="3" t="n">
         <v>20.3948757648468</v>
       </c>
-      <c r="L71" s="12" t="n">
+      <c r="L71" s="3" t="n">
         <v>24.8770549297333</v>
       </c>
-      <c r="M71" s="13" t="n">
+      <c r="M71" s="4" t="n">
         <v>0.0305691746613937</v>
       </c>
-      <c r="N71" s="13" t="n">
+      <c r="N71" s="4" t="n">
         <v>0.0280428825097413</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="0" t="s">
+      <c r="A72" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B72" s="0" t="s">
+      <c r="B72" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C72" s="0" t="n">
+      <c r="C72" s="1" t="n">
         <v>1041</v>
       </c>
-      <c r="D72" s="0" t="n">
+      <c r="D72" s="1" t="n">
         <v>462</v>
       </c>
-      <c r="E72" s="0" t="n">
+      <c r="E72" s="1" t="n">
         <v>480.942</v>
       </c>
-      <c r="F72" s="0" t="n">
-        <v>12</v>
-      </c>
-      <c r="G72" s="0" t="n">
-        <v>18</v>
-      </c>
-      <c r="H72" s="0" t="n">
-        <v>19</v>
-      </c>
-      <c r="I72" s="0" t="n">
-        <v>19</v>
-      </c>
-      <c r="J72" s="11" t="n">
+      <c r="F72" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="G72" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="H72" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="I72" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="J72" s="2" t="n">
         <v>0.08</v>
       </c>
-      <c r="K72" s="12" t="n">
+      <c r="K72" s="3" t="n">
         <v>20.3986096382141</v>
       </c>
-      <c r="L72" s="12" t="n">
+      <c r="L72" s="3" t="n">
         <v>25.7461357116699</v>
       </c>
-      <c r="M72" s="13" t="n">
+      <c r="M72" s="4" t="n">
         <v>0.0529253007639175</v>
       </c>
-      <c r="N72" s="13" t="n">
+      <c r="N72" s="4" t="n">
         <v>0.0478976674942093</v>
       </c>
     </row>
@@ -6860,90 +6919,90 @@
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="0" t="s">
+      <c r="A74" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B74" s="0" t="s">
+      <c r="B74" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C74" s="0" t="n">
+      <c r="C74" s="1" t="n">
         <v>1041</v>
       </c>
-      <c r="D74" s="0" t="n">
+      <c r="D74" s="1" t="n">
         <v>462</v>
       </c>
-      <c r="E74" s="0" t="n">
+      <c r="E74" s="1" t="n">
         <v>480.942</v>
       </c>
-      <c r="F74" s="0" t="n">
-        <v>12</v>
-      </c>
-      <c r="G74" s="0" t="n">
-        <v>18</v>
-      </c>
-      <c r="H74" s="0" t="n">
-        <v>19</v>
-      </c>
-      <c r="I74" s="0" t="n">
-        <v>19</v>
-      </c>
-      <c r="J74" s="11" t="n">
+      <c r="F74" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="G74" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="H74" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="I74" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="J74" s="2" t="n">
         <v>0.1</v>
       </c>
-      <c r="K74" s="12" t="n">
+      <c r="K74" s="3" t="n">
         <v>21.0117161273956</v>
       </c>
-      <c r="L74" s="12" t="n">
+      <c r="L74" s="3" t="n">
         <v>21.3067891597748</v>
       </c>
-      <c r="M74" s="13" t="n">
+      <c r="M74" s="4" t="n">
         <v>0.094244212399832</v>
       </c>
-      <c r="N74" s="13" t="n">
+      <c r="N74" s="4" t="n">
         <v>0.084586083145161</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="0" t="s">
+      <c r="A75" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B75" s="0" t="s">
+      <c r="B75" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C75" s="0" t="n">
+      <c r="C75" s="1" t="n">
         <v>1041</v>
       </c>
-      <c r="D75" s="0" t="n">
+      <c r="D75" s="1" t="n">
         <v>462</v>
       </c>
-      <c r="E75" s="0" t="n">
+      <c r="E75" s="1" t="n">
         <v>480.942</v>
       </c>
-      <c r="F75" s="0" t="n">
-        <v>12</v>
-      </c>
-      <c r="G75" s="0" t="n">
-        <v>18</v>
-      </c>
-      <c r="H75" s="0" t="n">
-        <v>19</v>
-      </c>
-      <c r="I75" s="0" t="n">
-        <v>19</v>
-      </c>
-      <c r="J75" s="11" t="n">
+      <c r="F75" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="G75" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="H75" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="I75" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="J75" s="2" t="n">
         <v>0.11</v>
       </c>
-      <c r="K75" s="12" t="n">
+      <c r="K75" s="3" t="n">
         <v>21.0975749492645</v>
       </c>
-      <c r="L75" s="12" t="n">
+      <c r="L75" s="3" t="n">
         <v>20.8536112308502</v>
       </c>
-      <c r="M75" s="13" t="n">
+      <c r="M75" s="4" t="n">
         <v>0.110185843615238</v>
       </c>
-      <c r="N75" s="13" t="n">
+      <c r="N75" s="4" t="n">
         <v>0.0980908300793027</v>
       </c>
     </row>
@@ -6992,90 +7051,90 @@
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="0" t="s">
+      <c r="A77" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B77" s="0" t="s">
+      <c r="B77" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C77" s="0" t="n">
+      <c r="C77" s="1" t="n">
         <v>1041</v>
       </c>
-      <c r="D77" s="0" t="n">
+      <c r="D77" s="1" t="n">
         <v>462</v>
       </c>
-      <c r="E77" s="0" t="n">
+      <c r="E77" s="1" t="n">
         <v>480.942</v>
       </c>
-      <c r="F77" s="0" t="n">
-        <v>12</v>
-      </c>
-      <c r="G77" s="0" t="n">
-        <v>18</v>
-      </c>
-      <c r="H77" s="0" t="n">
-        <v>19</v>
-      </c>
-      <c r="I77" s="0" t="n">
-        <v>19</v>
-      </c>
-      <c r="J77" s="11" t="n">
+      <c r="F77" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="G77" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="H77" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="I77" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="J77" s="2" t="n">
         <v>0.13</v>
       </c>
-      <c r="K77" s="12" t="n">
+      <c r="K77" s="3" t="n">
         <v>21.0367579460144</v>
       </c>
-      <c r="L77" s="12" t="n">
+      <c r="L77" s="3" t="n">
         <v>20.7206718921661</v>
       </c>
-      <c r="M77" s="13" t="n">
+      <c r="M77" s="4" t="n">
         <v>0.133315451759256</v>
       </c>
-      <c r="N77" s="13" t="n">
+      <c r="N77" s="4" t="n">
         <v>0.115577346124897</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="0" t="s">
+      <c r="A78" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B78" s="0" t="s">
+      <c r="B78" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C78" s="0" t="n">
+      <c r="C78" s="1" t="n">
         <v>1041</v>
       </c>
-      <c r="D78" s="0" t="n">
+      <c r="D78" s="1" t="n">
         <v>462</v>
       </c>
-      <c r="E78" s="0" t="n">
+      <c r="E78" s="1" t="n">
         <v>480.942</v>
       </c>
-      <c r="F78" s="0" t="n">
-        <v>12</v>
-      </c>
-      <c r="G78" s="0" t="n">
-        <v>18</v>
-      </c>
-      <c r="H78" s="0" t="n">
-        <v>19</v>
-      </c>
-      <c r="I78" s="0" t="n">
-        <v>19</v>
-      </c>
-      <c r="J78" s="11" t="n">
+      <c r="F78" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="G78" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="H78" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="I78" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="J78" s="2" t="n">
         <v>0.14</v>
       </c>
-      <c r="K78" s="12" t="n">
+      <c r="K78" s="3" t="n">
         <v>21.0888531208038</v>
       </c>
-      <c r="L78" s="12" t="n">
+      <c r="L78" s="3" t="n">
         <v>20.7450346946716</v>
       </c>
-      <c r="M78" s="13" t="n">
+      <c r="M78" s="4" t="n">
         <v>0.143759538572219</v>
       </c>
-      <c r="N78" s="13" t="n">
+      <c r="N78" s="4" t="n">
         <v>0.123272660736638</v>
       </c>
     </row>
@@ -8136,548 +8195,242 @@
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A103" s="0"/>
-      <c r="B103" s="0"/>
-      <c r="C103" s="0"/>
-      <c r="D103" s="0"/>
-      <c r="E103" s="0"/>
-      <c r="F103" s="0"/>
-      <c r="G103" s="0"/>
-      <c r="H103" s="0"/>
-      <c r="I103" s="0"/>
-      <c r="J103" s="0"/>
-      <c r="K103" s="0"/>
-      <c r="L103" s="0"/>
-      <c r="M103" s="0"/>
-      <c r="N103" s="0"/>
+      <c r="J103" s="1"/>
+      <c r="K103" s="1"/>
+      <c r="L103" s="1"/>
+      <c r="M103" s="1"/>
+      <c r="N103" s="1"/>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A104" s="0"/>
-      <c r="B104" s="0"/>
-      <c r="C104" s="0"/>
-      <c r="D104" s="0"/>
-      <c r="E104" s="0"/>
-      <c r="F104" s="0"/>
-      <c r="G104" s="0"/>
-      <c r="H104" s="0"/>
-      <c r="I104" s="0"/>
-      <c r="J104" s="0"/>
-      <c r="K104" s="0"/>
-      <c r="L104" s="0"/>
-      <c r="M104" s="0"/>
-      <c r="N104" s="0"/>
+      <c r="J104" s="1"/>
+      <c r="K104" s="1"/>
+      <c r="L104" s="1"/>
+      <c r="M104" s="1"/>
+      <c r="N104" s="1"/>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A105" s="0"/>
-      <c r="B105" s="0"/>
-      <c r="C105" s="0"/>
-      <c r="D105" s="0"/>
-      <c r="E105" s="0"/>
-      <c r="F105" s="0"/>
-      <c r="G105" s="0"/>
-      <c r="H105" s="0"/>
-      <c r="I105" s="0"/>
-      <c r="J105" s="0"/>
-      <c r="K105" s="0"/>
-      <c r="L105" s="0"/>
-      <c r="M105" s="0"/>
-      <c r="N105" s="0"/>
+      <c r="J105" s="1"/>
+      <c r="K105" s="1"/>
+      <c r="L105" s="1"/>
+      <c r="M105" s="1"/>
+      <c r="N105" s="1"/>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A106" s="0"/>
-      <c r="B106" s="0"/>
-      <c r="C106" s="0"/>
-      <c r="D106" s="0"/>
-      <c r="E106" s="0"/>
-      <c r="F106" s="0"/>
-      <c r="G106" s="0"/>
-      <c r="H106" s="0"/>
-      <c r="I106" s="0"/>
-      <c r="J106" s="0"/>
-      <c r="K106" s="0"/>
-      <c r="L106" s="0"/>
-      <c r="M106" s="0"/>
-      <c r="N106" s="0"/>
+      <c r="J106" s="1"/>
+      <c r="K106" s="1"/>
+      <c r="L106" s="1"/>
+      <c r="M106" s="1"/>
+      <c r="N106" s="1"/>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A107" s="0"/>
-      <c r="B107" s="0"/>
-      <c r="C107" s="0"/>
-      <c r="D107" s="0"/>
-      <c r="E107" s="0"/>
-      <c r="F107" s="0"/>
-      <c r="G107" s="0"/>
-      <c r="H107" s="0"/>
-      <c r="I107" s="0"/>
-      <c r="J107" s="0"/>
-      <c r="K107" s="0"/>
-      <c r="L107" s="0"/>
-      <c r="M107" s="0"/>
-      <c r="N107" s="0"/>
+      <c r="J107" s="1"/>
+      <c r="K107" s="1"/>
+      <c r="L107" s="1"/>
+      <c r="M107" s="1"/>
+      <c r="N107" s="1"/>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A108" s="0"/>
-      <c r="B108" s="0"/>
-      <c r="C108" s="0"/>
-      <c r="D108" s="0"/>
-      <c r="E108" s="0"/>
-      <c r="F108" s="0"/>
-      <c r="G108" s="0"/>
-      <c r="H108" s="0"/>
-      <c r="I108" s="0"/>
-      <c r="J108" s="0"/>
-      <c r="K108" s="0"/>
-      <c r="L108" s="0"/>
-      <c r="M108" s="0"/>
-      <c r="N108" s="0"/>
+      <c r="J108" s="1"/>
+      <c r="K108" s="1"/>
+      <c r="L108" s="1"/>
+      <c r="M108" s="1"/>
+      <c r="N108" s="1"/>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A109" s="0"/>
-      <c r="B109" s="0"/>
-      <c r="C109" s="0"/>
-      <c r="D109" s="0"/>
-      <c r="E109" s="0"/>
-      <c r="F109" s="0"/>
-      <c r="G109" s="0"/>
-      <c r="H109" s="0"/>
-      <c r="I109" s="0"/>
-      <c r="J109" s="0"/>
-      <c r="K109" s="0"/>
-      <c r="L109" s="0"/>
-      <c r="M109" s="0"/>
-      <c r="N109" s="0"/>
+      <c r="J109" s="1"/>
+      <c r="K109" s="1"/>
+      <c r="L109" s="1"/>
+      <c r="M109" s="1"/>
+      <c r="N109" s="1"/>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A110" s="0"/>
-      <c r="B110" s="0"/>
-      <c r="C110" s="0"/>
-      <c r="D110" s="0"/>
-      <c r="E110" s="0"/>
-      <c r="F110" s="0"/>
-      <c r="G110" s="0"/>
-      <c r="H110" s="0"/>
-      <c r="I110" s="0"/>
-      <c r="J110" s="0"/>
-      <c r="K110" s="0"/>
-      <c r="L110" s="0"/>
-      <c r="M110" s="0"/>
-      <c r="N110" s="0"/>
+      <c r="J110" s="1"/>
+      <c r="K110" s="1"/>
+      <c r="L110" s="1"/>
+      <c r="M110" s="1"/>
+      <c r="N110" s="1"/>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A111" s="0"/>
-      <c r="B111" s="0"/>
-      <c r="C111" s="0"/>
-      <c r="D111" s="0"/>
-      <c r="E111" s="0"/>
-      <c r="F111" s="0"/>
-      <c r="G111" s="0"/>
-      <c r="H111" s="0"/>
-      <c r="I111" s="0"/>
-      <c r="J111" s="0"/>
-      <c r="K111" s="0"/>
-      <c r="L111" s="0"/>
-      <c r="M111" s="0"/>
-      <c r="N111" s="0"/>
+      <c r="J111" s="1"/>
+      <c r="K111" s="1"/>
+      <c r="L111" s="1"/>
+      <c r="M111" s="1"/>
+      <c r="N111" s="1"/>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A112" s="0"/>
-      <c r="B112" s="0"/>
-      <c r="C112" s="0"/>
-      <c r="D112" s="0"/>
-      <c r="E112" s="0"/>
-      <c r="F112" s="0"/>
-      <c r="G112" s="0"/>
-      <c r="H112" s="0"/>
-      <c r="I112" s="0"/>
-      <c r="J112" s="0"/>
-      <c r="K112" s="0"/>
-      <c r="L112" s="0"/>
-      <c r="M112" s="0"/>
-      <c r="N112" s="0"/>
+      <c r="J112" s="1"/>
+      <c r="K112" s="1"/>
+      <c r="L112" s="1"/>
+      <c r="M112" s="1"/>
+      <c r="N112" s="1"/>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A113" s="0"/>
-      <c r="B113" s="0"/>
-      <c r="C113" s="0"/>
-      <c r="D113" s="0"/>
-      <c r="E113" s="0"/>
-      <c r="F113" s="0"/>
-      <c r="G113" s="0"/>
-      <c r="H113" s="0"/>
-      <c r="I113" s="0"/>
-      <c r="J113" s="0"/>
-      <c r="K113" s="0"/>
-      <c r="L113" s="0"/>
-      <c r="M113" s="0"/>
-      <c r="N113" s="0"/>
+      <c r="J113" s="1"/>
+      <c r="K113" s="1"/>
+      <c r="L113" s="1"/>
+      <c r="M113" s="1"/>
+      <c r="N113" s="1"/>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A114" s="0"/>
-      <c r="B114" s="0"/>
-      <c r="C114" s="0"/>
-      <c r="D114" s="0"/>
-      <c r="E114" s="0"/>
-      <c r="F114" s="0"/>
-      <c r="G114" s="0"/>
-      <c r="H114" s="0"/>
-      <c r="I114" s="0"/>
-      <c r="J114" s="0"/>
-      <c r="K114" s="0"/>
-      <c r="L114" s="0"/>
-      <c r="M114" s="0"/>
-      <c r="N114" s="0"/>
+      <c r="J114" s="1"/>
+      <c r="K114" s="1"/>
+      <c r="L114" s="1"/>
+      <c r="M114" s="1"/>
+      <c r="N114" s="1"/>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A115" s="0"/>
-      <c r="B115" s="0"/>
-      <c r="C115" s="0"/>
-      <c r="D115" s="0"/>
-      <c r="E115" s="0"/>
-      <c r="F115" s="0"/>
-      <c r="G115" s="0"/>
-      <c r="H115" s="0"/>
-      <c r="I115" s="0"/>
-      <c r="J115" s="0"/>
-      <c r="K115" s="0"/>
-      <c r="L115" s="0"/>
-      <c r="M115" s="0"/>
-      <c r="N115" s="0"/>
+      <c r="J115" s="1"/>
+      <c r="K115" s="1"/>
+      <c r="L115" s="1"/>
+      <c r="M115" s="1"/>
+      <c r="N115" s="1"/>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A116" s="0"/>
-      <c r="B116" s="0"/>
-      <c r="C116" s="0"/>
-      <c r="D116" s="0"/>
-      <c r="E116" s="0"/>
-      <c r="F116" s="0"/>
-      <c r="G116" s="0"/>
-      <c r="H116" s="0"/>
-      <c r="I116" s="0"/>
-      <c r="J116" s="0"/>
-      <c r="K116" s="0"/>
-      <c r="L116" s="0"/>
-      <c r="M116" s="0"/>
-      <c r="N116" s="0"/>
+      <c r="J116" s="1"/>
+      <c r="K116" s="1"/>
+      <c r="L116" s="1"/>
+      <c r="M116" s="1"/>
+      <c r="N116" s="1"/>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A117" s="0"/>
-      <c r="B117" s="0"/>
-      <c r="C117" s="0"/>
-      <c r="D117" s="0"/>
-      <c r="E117" s="0"/>
-      <c r="F117" s="0"/>
-      <c r="G117" s="0"/>
-      <c r="H117" s="0"/>
-      <c r="I117" s="0"/>
-      <c r="J117" s="0"/>
-      <c r="K117" s="0"/>
-      <c r="L117" s="0"/>
-      <c r="M117" s="0"/>
-      <c r="N117" s="0"/>
+      <c r="J117" s="1"/>
+      <c r="K117" s="1"/>
+      <c r="L117" s="1"/>
+      <c r="M117" s="1"/>
+      <c r="N117" s="1"/>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A118" s="0"/>
-      <c r="B118" s="0"/>
-      <c r="C118" s="0"/>
-      <c r="D118" s="0"/>
-      <c r="E118" s="0"/>
-      <c r="F118" s="0"/>
-      <c r="G118" s="0"/>
-      <c r="H118" s="0"/>
-      <c r="I118" s="0"/>
-      <c r="J118" s="0"/>
-      <c r="K118" s="0"/>
-      <c r="L118" s="0"/>
-      <c r="M118" s="0"/>
-      <c r="N118" s="0"/>
+      <c r="J118" s="1"/>
+      <c r="K118" s="1"/>
+      <c r="L118" s="1"/>
+      <c r="M118" s="1"/>
+      <c r="N118" s="1"/>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A119" s="0"/>
-      <c r="B119" s="0"/>
-      <c r="C119" s="0"/>
-      <c r="D119" s="0"/>
-      <c r="E119" s="0"/>
-      <c r="F119" s="0"/>
-      <c r="G119" s="0"/>
-      <c r="H119" s="0"/>
-      <c r="I119" s="0"/>
-      <c r="J119" s="0"/>
-      <c r="K119" s="0"/>
-      <c r="L119" s="0"/>
-      <c r="M119" s="0"/>
-      <c r="N119" s="0"/>
+      <c r="J119" s="1"/>
+      <c r="K119" s="1"/>
+      <c r="L119" s="1"/>
+      <c r="M119" s="1"/>
+      <c r="N119" s="1"/>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A120" s="0"/>
-      <c r="B120" s="0"/>
-      <c r="C120" s="0"/>
-      <c r="D120" s="0"/>
-      <c r="E120" s="0"/>
-      <c r="F120" s="0"/>
-      <c r="G120" s="0"/>
-      <c r="H120" s="0"/>
-      <c r="I120" s="0"/>
-      <c r="J120" s="0"/>
-      <c r="K120" s="0"/>
-      <c r="L120" s="0"/>
-      <c r="M120" s="0"/>
-      <c r="N120" s="0"/>
+      <c r="J120" s="1"/>
+      <c r="K120" s="1"/>
+      <c r="L120" s="1"/>
+      <c r="M120" s="1"/>
+      <c r="N120" s="1"/>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A121" s="0"/>
-      <c r="B121" s="0"/>
-      <c r="C121" s="0"/>
-      <c r="D121" s="0"/>
-      <c r="E121" s="0"/>
-      <c r="F121" s="0"/>
-      <c r="G121" s="0"/>
-      <c r="H121" s="0"/>
-      <c r="I121" s="0"/>
-      <c r="J121" s="0"/>
-      <c r="K121" s="0"/>
-      <c r="L121" s="0"/>
-      <c r="M121" s="0"/>
-      <c r="N121" s="0"/>
+      <c r="J121" s="1"/>
+      <c r="K121" s="1"/>
+      <c r="L121" s="1"/>
+      <c r="M121" s="1"/>
+      <c r="N121" s="1"/>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A122" s="0"/>
-      <c r="B122" s="0"/>
-      <c r="C122" s="0"/>
-      <c r="D122" s="0"/>
-      <c r="E122" s="0"/>
-      <c r="F122" s="0"/>
-      <c r="G122" s="0"/>
-      <c r="H122" s="0"/>
-      <c r="I122" s="0"/>
-      <c r="J122" s="0"/>
-      <c r="K122" s="0"/>
-      <c r="L122" s="0"/>
-      <c r="M122" s="0"/>
-      <c r="N122" s="0"/>
+      <c r="J122" s="1"/>
+      <c r="K122" s="1"/>
+      <c r="L122" s="1"/>
+      <c r="M122" s="1"/>
+      <c r="N122" s="1"/>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A123" s="0"/>
-      <c r="B123" s="0"/>
-      <c r="C123" s="0"/>
-      <c r="D123" s="0"/>
-      <c r="E123" s="0"/>
-      <c r="F123" s="0"/>
-      <c r="G123" s="0"/>
-      <c r="H123" s="0"/>
-      <c r="I123" s="0"/>
-      <c r="J123" s="0"/>
-      <c r="K123" s="0"/>
-      <c r="L123" s="0"/>
-      <c r="M123" s="0"/>
-      <c r="N123" s="0"/>
+      <c r="J123" s="1"/>
+      <c r="K123" s="1"/>
+      <c r="L123" s="1"/>
+      <c r="M123" s="1"/>
+      <c r="N123" s="1"/>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A124" s="0"/>
-      <c r="B124" s="0"/>
-      <c r="C124" s="0"/>
-      <c r="D124" s="0"/>
-      <c r="E124" s="0"/>
-      <c r="F124" s="0"/>
-      <c r="G124" s="0"/>
-      <c r="H124" s="0"/>
-      <c r="I124" s="0"/>
-      <c r="J124" s="0"/>
-      <c r="K124" s="0"/>
-      <c r="L124" s="0"/>
-      <c r="M124" s="0"/>
-      <c r="N124" s="0"/>
+      <c r="J124" s="1"/>
+      <c r="K124" s="1"/>
+      <c r="L124" s="1"/>
+      <c r="M124" s="1"/>
+      <c r="N124" s="1"/>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A125" s="0"/>
-      <c r="B125" s="0"/>
-      <c r="C125" s="0"/>
-      <c r="D125" s="0"/>
-      <c r="E125" s="0"/>
-      <c r="F125" s="0"/>
-      <c r="G125" s="0"/>
-      <c r="H125" s="0"/>
-      <c r="I125" s="0"/>
-      <c r="J125" s="0"/>
-      <c r="K125" s="0"/>
-      <c r="L125" s="0"/>
-      <c r="M125" s="0"/>
-      <c r="N125" s="0"/>
+      <c r="J125" s="1"/>
+      <c r="K125" s="1"/>
+      <c r="L125" s="1"/>
+      <c r="M125" s="1"/>
+      <c r="N125" s="1"/>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A126" s="0"/>
-      <c r="B126" s="0"/>
-      <c r="C126" s="0"/>
-      <c r="D126" s="0"/>
-      <c r="E126" s="0"/>
-      <c r="F126" s="0"/>
-      <c r="G126" s="0"/>
-      <c r="H126" s="0"/>
-      <c r="I126" s="0"/>
-      <c r="J126" s="0"/>
-      <c r="K126" s="0"/>
-      <c r="L126" s="0"/>
-      <c r="M126" s="0"/>
-      <c r="N126" s="0"/>
+      <c r="J126" s="1"/>
+      <c r="K126" s="1"/>
+      <c r="L126" s="1"/>
+      <c r="M126" s="1"/>
+      <c r="N126" s="1"/>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A127" s="0"/>
-      <c r="B127" s="0"/>
-      <c r="C127" s="0"/>
-      <c r="D127" s="0"/>
-      <c r="E127" s="0"/>
-      <c r="F127" s="0"/>
-      <c r="G127" s="0"/>
-      <c r="H127" s="0"/>
-      <c r="I127" s="0"/>
-      <c r="J127" s="0"/>
-      <c r="K127" s="0"/>
-      <c r="L127" s="0"/>
-      <c r="M127" s="0"/>
-      <c r="N127" s="0"/>
+      <c r="J127" s="1"/>
+      <c r="K127" s="1"/>
+      <c r="L127" s="1"/>
+      <c r="M127" s="1"/>
+      <c r="N127" s="1"/>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A128" s="0"/>
-      <c r="B128" s="0"/>
-      <c r="C128" s="0"/>
-      <c r="D128" s="0"/>
-      <c r="E128" s="0"/>
-      <c r="F128" s="0"/>
-      <c r="G128" s="0"/>
-      <c r="H128" s="0"/>
-      <c r="I128" s="0"/>
-      <c r="J128" s="0"/>
-      <c r="K128" s="0"/>
-      <c r="L128" s="0"/>
-      <c r="M128" s="0"/>
-      <c r="N128" s="0"/>
+      <c r="J128" s="1"/>
+      <c r="K128" s="1"/>
+      <c r="L128" s="1"/>
+      <c r="M128" s="1"/>
+      <c r="N128" s="1"/>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A129" s="0"/>
-      <c r="B129" s="0"/>
-      <c r="C129" s="0"/>
-      <c r="D129" s="0"/>
-      <c r="E129" s="0"/>
-      <c r="F129" s="0"/>
-      <c r="G129" s="0"/>
-      <c r="H129" s="0"/>
-      <c r="I129" s="0"/>
-      <c r="J129" s="0"/>
-      <c r="K129" s="0"/>
-      <c r="L129" s="0"/>
-      <c r="M129" s="0"/>
-      <c r="N129" s="0"/>
+      <c r="J129" s="1"/>
+      <c r="K129" s="1"/>
+      <c r="L129" s="1"/>
+      <c r="M129" s="1"/>
+      <c r="N129" s="1"/>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A130" s="0"/>
-      <c r="B130" s="0"/>
-      <c r="C130" s="0"/>
-      <c r="D130" s="0"/>
-      <c r="E130" s="0"/>
-      <c r="F130" s="0"/>
-      <c r="G130" s="0"/>
-      <c r="H130" s="0"/>
-      <c r="I130" s="0"/>
-      <c r="J130" s="0"/>
-      <c r="K130" s="0"/>
-      <c r="L130" s="0"/>
-      <c r="M130" s="0"/>
-      <c r="N130" s="0"/>
+      <c r="J130" s="1"/>
+      <c r="K130" s="1"/>
+      <c r="L130" s="1"/>
+      <c r="M130" s="1"/>
+      <c r="N130" s="1"/>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A131" s="0"/>
-      <c r="B131" s="0"/>
-      <c r="C131" s="0"/>
-      <c r="D131" s="0"/>
-      <c r="E131" s="0"/>
-      <c r="F131" s="0"/>
-      <c r="G131" s="0"/>
-      <c r="H131" s="0"/>
-      <c r="I131" s="0"/>
-      <c r="J131" s="0"/>
-      <c r="K131" s="0"/>
-      <c r="L131" s="0"/>
-      <c r="M131" s="0"/>
-      <c r="N131" s="0"/>
+      <c r="J131" s="1"/>
+      <c r="K131" s="1"/>
+      <c r="L131" s="1"/>
+      <c r="M131" s="1"/>
+      <c r="N131" s="1"/>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A132" s="0"/>
-      <c r="B132" s="0"/>
-      <c r="C132" s="0"/>
-      <c r="D132" s="0"/>
-      <c r="E132" s="0"/>
-      <c r="F132" s="0"/>
-      <c r="G132" s="0"/>
-      <c r="H132" s="0"/>
-      <c r="I132" s="0"/>
-      <c r="J132" s="0"/>
-      <c r="K132" s="0"/>
-      <c r="L132" s="0"/>
-      <c r="M132" s="0"/>
-      <c r="N132" s="0"/>
+      <c r="J132" s="1"/>
+      <c r="K132" s="1"/>
+      <c r="L132" s="1"/>
+      <c r="M132" s="1"/>
+      <c r="N132" s="1"/>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A133" s="0"/>
-      <c r="B133" s="0"/>
-      <c r="C133" s="0"/>
-      <c r="D133" s="0"/>
-      <c r="E133" s="0"/>
-      <c r="F133" s="0"/>
-      <c r="G133" s="0"/>
-      <c r="H133" s="0"/>
-      <c r="I133" s="0"/>
-      <c r="J133" s="0"/>
-      <c r="K133" s="0"/>
-      <c r="L133" s="0"/>
-      <c r="M133" s="0"/>
-      <c r="N133" s="0"/>
+      <c r="J133" s="1"/>
+      <c r="K133" s="1"/>
+      <c r="L133" s="1"/>
+      <c r="M133" s="1"/>
+      <c r="N133" s="1"/>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A134" s="0"/>
-      <c r="B134" s="0"/>
-      <c r="C134" s="0"/>
-      <c r="D134" s="0"/>
-      <c r="E134" s="0"/>
-      <c r="F134" s="0"/>
-      <c r="G134" s="0"/>
-      <c r="H134" s="0"/>
-      <c r="I134" s="0"/>
-      <c r="J134" s="0"/>
-      <c r="K134" s="0"/>
-      <c r="L134" s="0"/>
-      <c r="M134" s="0"/>
-      <c r="N134" s="0"/>
+      <c r="J134" s="1"/>
+      <c r="K134" s="1"/>
+      <c r="L134" s="1"/>
+      <c r="M134" s="1"/>
+      <c r="N134" s="1"/>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A135" s="0"/>
-      <c r="B135" s="0"/>
-      <c r="C135" s="0"/>
-      <c r="D135" s="0"/>
-      <c r="E135" s="0"/>
-      <c r="F135" s="0"/>
-      <c r="G135" s="0"/>
-      <c r="H135" s="0"/>
-      <c r="I135" s="0"/>
-      <c r="J135" s="0"/>
-      <c r="K135" s="0"/>
-      <c r="L135" s="0"/>
-      <c r="M135" s="0"/>
-      <c r="N135" s="0"/>
+      <c r="J135" s="1"/>
+      <c r="K135" s="1"/>
+      <c r="L135" s="1"/>
+      <c r="M135" s="1"/>
+      <c r="N135" s="1"/>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A136" s="0"/>
-      <c r="B136" s="0"/>
-      <c r="C136" s="0"/>
-      <c r="D136" s="0"/>
-      <c r="E136" s="0"/>
-      <c r="F136" s="0"/>
-      <c r="G136" s="0"/>
-      <c r="H136" s="0"/>
-      <c r="I136" s="0"/>
-      <c r="J136" s="0"/>
-      <c r="K136" s="0"/>
-      <c r="L136" s="0"/>
-      <c r="M136" s="0"/>
-      <c r="N136" s="0"/>
+      <c r="J136" s="1"/>
+      <c r="K136" s="1"/>
+      <c r="L136" s="1"/>
+      <c r="M136" s="1"/>
+      <c r="N136" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
meilleure qualité pour les graphiques et réorganisation
</commit_message>
<xml_diff>
--- a/excel/résultats.xlsx
+++ b/excel/résultats.xlsx
@@ -802,11 +802,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="97839022"/>
-        <c:axId val="59265966"/>
+        <c:axId val="35116449"/>
+        <c:axId val="94909323"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="97839022"/>
+        <c:axId val="35116449"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -871,12 +871,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="59265966"/>
+        <c:crossAx val="94909323"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="59265966"/>
+        <c:axId val="94909323"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -950,7 +950,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="97839022"/>
+        <c:crossAx val="35116449"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1401,11 +1401,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="94585710"/>
-        <c:axId val="37454558"/>
+        <c:axId val="48722969"/>
+        <c:axId val="95923396"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="94585710"/>
+        <c:axId val="48722969"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1470,12 +1470,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="37454558"/>
+        <c:crossAx val="95923396"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="37454558"/>
+        <c:axId val="95923396"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1549,7 +1549,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94585710"/>
+        <c:crossAx val="48722969"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1993,11 +1993,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="84307685"/>
-        <c:axId val="81840256"/>
+        <c:axId val="77635731"/>
+        <c:axId val="3088897"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="84307685"/>
+        <c:axId val="77635731"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2062,12 +2062,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="81840256"/>
+        <c:crossAx val="3088897"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="81840256"/>
+        <c:axId val="3088897"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2141,7 +2141,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="84307685"/>
+        <c:crossAx val="77635731"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2324,8 +2324,8 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="30331516"/>
-        <c:axId val="97602717"/>
+        <c:axId val="47442075"/>
+        <c:axId val="2081877"/>
       </c:scatterChart>
       <c:scatterChart>
         <c:scatterStyle val="lineMarker"/>
@@ -2443,11 +2443,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="14661021"/>
-        <c:axId val="61472382"/>
+        <c:axId val="21566347"/>
+        <c:axId val="2309860"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="30331516"/>
+        <c:axId val="47442075"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2512,12 +2512,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="97602717"/>
+        <c:crossAx val="2081877"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="97602717"/>
+        <c:axId val="2081877"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2591,12 +2591,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="30331516"/>
+        <c:crossAx val="47442075"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="14661021"/>
+        <c:axId val="21566347"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2628,11 +2628,11 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="61472382"/>
+        <c:crossAx val="2309860"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="61472382"/>
+        <c:axId val="2309860"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2697,7 +2697,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="14661021"/>
+        <c:crossAx val="21566347"/>
         <c:crosses val="max"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2916,8 +2916,8 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="17542930"/>
-        <c:axId val="78239994"/>
+        <c:axId val="47845381"/>
+        <c:axId val="69909783"/>
       </c:scatterChart>
       <c:scatterChart>
         <c:scatterStyle val="lineMarker"/>
@@ -3071,11 +3071,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="5242227"/>
-        <c:axId val="7148327"/>
+        <c:axId val="37957100"/>
+        <c:axId val="71328613"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="17542930"/>
+        <c:axId val="47845381"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3140,12 +3140,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="78239994"/>
+        <c:crossAx val="69909783"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="78239994"/>
+        <c:axId val="69909783"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3219,12 +3219,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="17542930"/>
+        <c:crossAx val="47845381"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="5242227"/>
+        <c:axId val="37957100"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3256,11 +3256,11 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="7148327"/>
+        <c:crossAx val="71328613"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="7148327"/>
+        <c:axId val="71328613"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3325,7 +3325,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="5242227"/>
+        <c:crossAx val="37957100"/>
         <c:crosses val="max"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -3363,9 +3363,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>25</xdr:col>
-      <xdr:colOff>168840</xdr:colOff>
+      <xdr:colOff>168480</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>6840</xdr:rowOff>
+      <xdr:rowOff>6480</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3374,7 +3374,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="10048680" y="81720"/>
-        <a:ext cx="6652440" cy="3544560"/>
+        <a:ext cx="6652080" cy="3544200"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3393,9 +3393,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>25</xdr:col>
-      <xdr:colOff>260280</xdr:colOff>
+      <xdr:colOff>259920</xdr:colOff>
       <xdr:row>38</xdr:row>
-      <xdr:rowOff>156600</xdr:rowOff>
+      <xdr:rowOff>156240</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3404,7 +3404,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="10083960" y="3714840"/>
-        <a:ext cx="6708600" cy="3680640"/>
+        <a:ext cx="6708240" cy="3680280"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3423,9 +3423,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>26</xdr:col>
-      <xdr:colOff>147240</xdr:colOff>
+      <xdr:colOff>146880</xdr:colOff>
       <xdr:row>60</xdr:row>
-      <xdr:rowOff>6840</xdr:rowOff>
+      <xdr:rowOff>6480</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3434,7 +3434,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="10040040" y="7483680"/>
-        <a:ext cx="7327080" cy="3953160"/>
+        <a:ext cx="7326720" cy="3952800"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3453,9 +3453,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>26</xdr:col>
-      <xdr:colOff>340560</xdr:colOff>
+      <xdr:colOff>340200</xdr:colOff>
       <xdr:row>83</xdr:row>
-      <xdr:rowOff>41400</xdr:rowOff>
+      <xdr:rowOff>41040</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3464,7 +3464,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="10085400" y="11648160"/>
-        <a:ext cx="7475040" cy="4204800"/>
+        <a:ext cx="7474680" cy="4204440"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3483,9 +3483,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>26</xdr:col>
-      <xdr:colOff>380880</xdr:colOff>
+      <xdr:colOff>380520</xdr:colOff>
       <xdr:row>105</xdr:row>
-      <xdr:rowOff>20160</xdr:rowOff>
+      <xdr:rowOff>19800</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3494,7 +3494,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="10111680" y="16111080"/>
-        <a:ext cx="7489080" cy="3911760"/>
+        <a:ext cx="7488720" cy="3911400"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">

</xml_diff>